<commit_message>
Warehouse Diff locations same item
</commit_message>
<xml_diff>
--- a/public/warehouse/item_warehouse.xlsx
+++ b/public/warehouse/item_warehouse.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Atul kumar\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_96BB3AF33AA4EF5CD49BA13D9F61BCA0E405F18A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Item Warehouse" sheetId="1" r:id="rId1"/>
@@ -14,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
   <si>
     <t>item_code</t>
   </si>
@@ -31,72 +37,78 @@
     <t>TY-122-K</t>
   </si>
   <si>
-    <t>SF169-62-30</t>
+    <t>R1-1-3</t>
   </si>
   <si>
     <t>TY-280-S</t>
   </si>
   <si>
-    <t>R28-34-60</t>
+    <t>R1-2-1</t>
   </si>
   <si>
     <t>TY-561-S</t>
   </si>
   <si>
-    <t>R9-52-30</t>
+    <t>R1-4-1</t>
   </si>
   <si>
     <t>TY-572-N</t>
   </si>
   <si>
-    <t>R30-14-50</t>
+    <t>R1-6-6</t>
   </si>
   <si>
     <t>TY-053-T</t>
   </si>
   <si>
-    <t>R10-40-10</t>
+    <t>R4-1-6</t>
   </si>
   <si>
     <t>TY-001-A</t>
   </si>
   <si>
-    <t>FF140-10-60</t>
+    <t>R4-6-5</t>
   </si>
   <si>
     <t>TY-113-E</t>
   </si>
   <si>
-    <t>R5-27-10</t>
+    <t>R5-2-5</t>
   </si>
   <si>
     <t>TY-059-M</t>
   </si>
   <si>
-    <t>TF182-71-40</t>
+    <t>R10-23-6</t>
   </si>
   <si>
     <t>TY-126-D</t>
   </si>
   <si>
-    <t>GF115-57-50</t>
+    <t>R11-4-3</t>
   </si>
   <si>
     <t>TY-221-M</t>
   </si>
   <si>
-    <t>GF103-30-60</t>
+    <t>R12-25-4</t>
+  </si>
+  <si>
+    <t>R2-2-5</t>
+  </si>
+  <si>
+    <t>R2-1-2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -122,15 +134,19 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -432,12 +448,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main">
-  <sheetPr/>
-  <dimension ref="A1:D11"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -451,7 +466,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -465,7 +480,7 @@
         <v>46007</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -479,7 +494,7 @@
         <v>45998</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -493,7 +508,7 @@
         <v>46015</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -507,7 +522,7 @@
         <v>46067</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -521,7 +536,7 @@
         <v>46076</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -535,7 +550,7 @@
         <v>46042</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -549,7 +564,7 @@
         <v>46043</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -563,7 +578,7 @@
         <v>46017</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -577,7 +592,7 @@
         <v>46045</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -591,8 +606,36 @@
         <v>46016</v>
       </c>
     </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12">
+        <v>16</v>
+      </c>
+      <c r="D12" s="1">
+        <v>46096.770833333336</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13">
+        <v>10</v>
+      </c>
+      <c r="D13" s="1">
+        <v>46096.770833333336</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup orientation="portrait" scale="100" paperSize="9" fitToWidth="0" fitToHeight="0" horizontalDpi="0" verticalDpi="0" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>